<commit_message>
Added a little more on loot boxes into GDV4000 Ethics
</commit_message>
<xml_diff>
--- a/T1/GDV5000/Teams_25.xlsx
+++ b/T1/GDV5000/Teams_25.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\T1\GDV5000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85BDC46D-F369-4E11-91F8-4A6112BA5820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3865A63C-7271-4E90-A1E1-5AA86CD6A397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{9DBA8AA2-FEE3-408C-9D13-BB1908EF39A4}"/>
+    <workbookView xWindow="3072" yWindow="3072" windowWidth="34560" windowHeight="18600" xr2:uid="{9DBA8AA2-FEE3-408C-9D13-BB1908EF39A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -195,7 +195,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -207,6 +207,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -245,7 +252,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -265,6 +272,19 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -744,25 +764,25 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="7">
-        <v>0.4</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="E8" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="F8" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G8" s="8">
-        <v>0.6</v>
-      </c>
-      <c r="H8" s="4" t="s">
+      <c r="G8" s="12">
+        <v>0.6</v>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>